<commit_message>
Replace all em dashes with hyphens, sync from main
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VCCorner_Template_v2.xlsx
+++ b/VCCorner_Template_v2.xlsx
@@ -741,7 +741,7 @@
       <c r="A2" s="44" t="n"/>
       <c r="B2" s="45" t="inlineStr">
         <is>
-          <t>THE VC CORNER — Quick Start Guide</t>
+          <t>THE VC CORNER - Quick Start Guide</t>
         </is>
       </c>
     </row>
@@ -815,7 +815,7 @@
       <c r="A12" s="44" t="n"/>
       <c r="B12" s="46" t="inlineStr">
         <is>
-          <t>Open the sheet matching your Business Type (AI-SaaS, D2C, or Healthcare). Fill only the blue cells — these are your inputs. Gray cells with formulas will auto-calculate. Enter 5-year projections in columns B through F.</t>
+          <t>Open the sheet matching your Business Type (AI-SaaS, D2C, or Healthcare). Fill only the blue cells - these are your inputs. Gray cells with formulas will auto-calculate. Enter 5-year projections in columns B through F.</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       <c r="A15" s="44" t="n"/>
       <c r="B15" s="46" t="inlineStr">
         <is>
-          <t>Save this file, then go to thevcorner.com. Click 'Upload Template' and select your saved .xlsx file. Everything runs in your browser — your data never leaves your device.</t>
+          <t>Save this file, then go to thevcorner.com. Click 'Upload Template' and select your saved .xlsx file. Everything runs in your browser - your data never leaves your device.</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="C22" s="50" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Your input — fill these cells</t>
+          <t xml:space="preserve">  Your input - fill these cells</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
       </c>
       <c r="C23" s="50" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Auto-calculated (formula) — do not edit</t>
+          <t xml:space="preserve">  Auto-calculated (formula) - do not edit</t>
         </is>
       </c>
     </row>
@@ -940,7 +940,7 @@
       <c r="A27" s="44" t="n"/>
       <c r="B27" s="53" t="inlineStr">
         <is>
-          <t xml:space="preserve">  •  Only fill sections you marked 'Yes' on the Checklist — everything else is ignored.</t>
+          <t xml:space="preserve">  •  Only fill sections you marked 'Yes' on the Checklist - everything else is ignored.</t>
         </is>
       </c>
     </row>
@@ -964,7 +964,7 @@
       <c r="A30" s="44" t="n"/>
       <c r="B30" s="53" t="inlineStr">
         <is>
-          <t xml:space="preserve">  •  Upload your completed file at thevcorner.com — 100% private, browser-only processing.</t>
+          <t xml:space="preserve">  •  Upload your completed file at thevcorner.com - 100% private, browser-only processing.</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>THE VC CORNER — Company Setup</t>
+          <t>THE VC CORNER - Company Setup</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>THE VC CORNER — Section Checklist</t>
+          <t>THE VC CORNER - Section Checklist</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
 • Set each section to Yes or No
 • Only 'Yes' sections appear on the dashboard
 • The original 10 sections per sector default to Yes
-• New v2 sections default to No — enable as needed</t>
+• New v2 sections default to No - enable as needed</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>THE VC CORNER — AI-SaaS Projections</t>
+          <t>THE VC CORNER - AI-SaaS Projections</t>
         </is>
       </c>
     </row>
@@ -5766,7 +5766,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>THE VC CORNER — D2C Projections</t>
+          <t>THE VC CORNER - D2C Projections</t>
         </is>
       </c>
     </row>
@@ -5892,7 +5892,7 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  GMV — Website</t>
+          <t xml:space="preserve">  GMV - Website</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -5987,7 +5987,7 @@
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  GMV — Retail</t>
+          <t xml:space="preserve">  GMV - Retail</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -6082,7 +6082,7 @@
     <row r="19">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  GMV — Marketplace</t>
+          <t xml:space="preserve">  GMV - Marketplace</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -6184,7 +6184,7 @@
     <row r="24">
       <c r="A24" s="17" t="inlineStr">
         <is>
-          <t>Website — GMV</t>
+          <t>Website - GMV</t>
         </is>
       </c>
       <c r="B24" s="18" t="n"/>
@@ -6201,7 +6201,7 @@
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
         <is>
-          <t>Website — Return Rate</t>
+          <t>Website - Return Rate</t>
         </is>
       </c>
       <c r="B25" s="27" t="n"/>
@@ -6218,7 +6218,7 @@
     <row r="26">
       <c r="A26" s="19" t="inlineStr">
         <is>
-          <t>Website — Net Revenue</t>
+          <t>Website - Net Revenue</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -6250,7 +6250,7 @@
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>Retail — GMV</t>
+          <t>Retail - GMV</t>
         </is>
       </c>
       <c r="B27" s="18" t="n"/>
@@ -6267,7 +6267,7 @@
     <row r="28">
       <c r="A28" s="17" t="inlineStr">
         <is>
-          <t>Retail — Return Rate</t>
+          <t>Retail - Return Rate</t>
         </is>
       </c>
       <c r="B28" s="27" t="n"/>
@@ -6284,7 +6284,7 @@
     <row r="29">
       <c r="A29" s="19" t="inlineStr">
         <is>
-          <t>Retail — Net Revenue</t>
+          <t>Retail - Net Revenue</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -6316,7 +6316,7 @@
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>Marketplace — GMV</t>
+          <t>Marketplace - GMV</t>
         </is>
       </c>
       <c r="B30" s="18" t="n"/>
@@ -6333,7 +6333,7 @@
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>Marketplace — Return Rate</t>
+          <t>Marketplace - Return Rate</t>
         </is>
       </c>
       <c r="B31" s="27" t="n"/>
@@ -6350,7 +6350,7 @@
     <row r="32">
       <c r="A32" s="17" t="inlineStr">
         <is>
-          <t>Marketplace — Commission %</t>
+          <t>Marketplace - Commission %</t>
         </is>
       </c>
       <c r="B32" s="27" t="n"/>
@@ -6367,7 +6367,7 @@
     <row r="33">
       <c r="A33" s="19" t="inlineStr">
         <is>
-          <t>Marketplace — Net Revenue</t>
+          <t>Marketplace - Net Revenue</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -6452,7 +6452,7 @@
     <row r="37">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>Website — Gross Revenue</t>
+          <t>Website - Gross Revenue</t>
         </is>
       </c>
       <c r="B37" s="18" t="n"/>
@@ -6469,7 +6469,7 @@
     <row r="38">
       <c r="A38" s="17" t="inlineStr">
         <is>
-          <t>Website — Returns</t>
+          <t>Website - Returns</t>
         </is>
       </c>
       <c r="B38" s="18" t="n"/>
@@ -6486,7 +6486,7 @@
     <row r="39">
       <c r="A39" s="19" t="inlineStr">
         <is>
-          <t>Website — Net Revenue</t>
+          <t>Website - Net Revenue</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -6518,7 +6518,7 @@
     <row r="40">
       <c r="A40" s="17" t="inlineStr">
         <is>
-          <t>Retail — Gross Revenue</t>
+          <t>Retail - Gross Revenue</t>
         </is>
       </c>
       <c r="B40" s="18" t="n"/>
@@ -6535,7 +6535,7 @@
     <row r="41">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>Retail — Returns</t>
+          <t>Retail - Returns</t>
         </is>
       </c>
       <c r="B41" s="18" t="n"/>
@@ -6552,7 +6552,7 @@
     <row r="42">
       <c r="A42" s="19" t="inlineStr">
         <is>
-          <t>Retail — Net Revenue</t>
+          <t>Retail - Net Revenue</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -6584,7 +6584,7 @@
     <row r="43">
       <c r="A43" s="17" t="inlineStr">
         <is>
-          <t>Marketplace — Gross Revenue</t>
+          <t>Marketplace - Gross Revenue</t>
         </is>
       </c>
       <c r="B43" s="18" t="n"/>
@@ -6601,7 +6601,7 @@
     <row r="44">
       <c r="A44" s="17" t="inlineStr">
         <is>
-          <t>Marketplace — Returns</t>
+          <t>Marketplace - Returns</t>
         </is>
       </c>
       <c r="B44" s="18" t="n"/>
@@ -6618,7 +6618,7 @@
     <row r="45">
       <c r="A45" s="17" t="inlineStr">
         <is>
-          <t>Marketplace — Commission</t>
+          <t>Marketplace - Commission</t>
         </is>
       </c>
       <c r="B45" s="18" t="n"/>
@@ -6635,7 +6635,7 @@
     <row r="46">
       <c r="A46" s="19" t="inlineStr">
         <is>
-          <t>Marketplace — Net Revenue</t>
+          <t>Marketplace - Net Revenue</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -6841,7 +6841,7 @@
     <row r="57">
       <c r="A57" s="17" t="inlineStr">
         <is>
-          <t>Website — Churn Rate</t>
+          <t>Website - Churn Rate</t>
         </is>
       </c>
       <c r="B57" s="27" t="n"/>
@@ -6858,7 +6858,7 @@
     <row r="58">
       <c r="A58" s="17" t="inlineStr">
         <is>
-          <t>Retail — Churn Rate</t>
+          <t>Retail - Churn Rate</t>
         </is>
       </c>
       <c r="B58" s="27" t="n"/>
@@ -6875,7 +6875,7 @@
     <row r="59">
       <c r="A59" s="17" t="inlineStr">
         <is>
-          <t>Marketplace — Churn Rate</t>
+          <t>Marketplace - Churn Rate</t>
         </is>
       </c>
       <c r="B59" s="27" t="n"/>
@@ -9101,7 +9101,7 @@
     <row r="181">
       <c r="A181" s="17" t="inlineStr">
         <is>
-          <t>Website — Revenue</t>
+          <t>Website - Revenue</t>
         </is>
       </c>
       <c r="B181" s="18" t="n"/>
@@ -9118,7 +9118,7 @@
     <row r="182">
       <c r="A182" s="17" t="inlineStr">
         <is>
-          <t>Website — Variable Cost</t>
+          <t>Website - Variable Cost</t>
         </is>
       </c>
       <c r="B182" s="18" t="n"/>
@@ -9135,7 +9135,7 @@
     <row r="183">
       <c r="A183" s="19" t="inlineStr">
         <is>
-          <t>Website — Contribution Margin</t>
+          <t>Website - Contribution Margin</t>
         </is>
       </c>
       <c r="B183" s="20">
@@ -9167,7 +9167,7 @@
     <row r="184">
       <c r="A184" s="17" t="inlineStr">
         <is>
-          <t>Retail — Revenue</t>
+          <t>Retail - Revenue</t>
         </is>
       </c>
       <c r="B184" s="18" t="n"/>
@@ -9184,7 +9184,7 @@
     <row r="185">
       <c r="A185" s="17" t="inlineStr">
         <is>
-          <t>Retail — Variable Cost</t>
+          <t>Retail - Variable Cost</t>
         </is>
       </c>
       <c r="B185" s="18" t="n"/>
@@ -9201,7 +9201,7 @@
     <row r="186">
       <c r="A186" s="19" t="inlineStr">
         <is>
-          <t>Retail — Contribution Margin</t>
+          <t>Retail - Contribution Margin</t>
         </is>
       </c>
       <c r="B186" s="20">
@@ -9233,7 +9233,7 @@
     <row r="187">
       <c r="A187" s="17" t="inlineStr">
         <is>
-          <t>Marketplace — Revenue</t>
+          <t>Marketplace - Revenue</t>
         </is>
       </c>
       <c r="B187" s="18" t="n"/>
@@ -9250,7 +9250,7 @@
     <row r="188">
       <c r="A188" s="17" t="inlineStr">
         <is>
-          <t>Marketplace — Variable Cost</t>
+          <t>Marketplace - Variable Cost</t>
         </is>
       </c>
       <c r="B188" s="18" t="n"/>
@@ -9267,7 +9267,7 @@
     <row r="189">
       <c r="A189" s="19" t="inlineStr">
         <is>
-          <t>Marketplace — Contribution Margin</t>
+          <t>Marketplace - Contribution Margin</t>
         </is>
       </c>
       <c r="B189" s="20">
@@ -9714,7 +9714,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>THE VC CORNER — Healthcare Projections</t>
+          <t>THE VC CORNER - Healthcare Projections</t>
         </is>
       </c>
     </row>

</xml_diff>